<commit_message>
Composição visual: QEF com EC2, EC5 e limites afinados
- Notas: a coluna de preenchimento é a amarela (J), não a azul
- EC2: conta os 3 pares seguidos de tamanhos com razão ≥ 1,2
- EC5: proporção 2:1, espaço vazio do lado do texto e perceção do
  equilíbrio no teste com utilizadores (pergunta nova nas Notas)
- E03 e FC4: limites sem sobreposições nem buracos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Files/Teoricas/ComposicaoVisual_QEF_Grupo1.xlsx
+++ b/Files/Teoricas/ComposicaoVisual_QEF_Grupo1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tiago\AppData\Local\Temp\claude\C--Users-tiago-Desktop-Mestrado-2Ano-CAMUL-RepoCamul-CAMUL-2026\67b76cae-61ff-4d41-a191-a6d9f77c0f89\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB3FD362-5C65-4475-AE18-1EC62635A4DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E86D98A-5DCE-4E56-8EF4-37B2C1776948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2BE1A5F0-6062-45CC-8E94-69B694959B5C}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="210">
   <si>
     <t>q (%)</t>
   </si>
@@ -316,12 +316,6 @@
     <t>0–3</t>
   </si>
   <si>
-    <t>4–5</t>
-  </si>
-  <si>
-    <t>6–7</t>
-  </si>
-  <si>
     <t>Teste com utilizadores (ver Notas)</t>
   </si>
   <si>
@@ -358,12 +352,6 @@
     <t>&gt; 10 s</t>
   </si>
   <si>
-    <t>6–10 s</t>
-  </si>
-  <si>
-    <t>3–6 s</t>
-  </si>
-  <si>
     <t>2–3 s</t>
   </si>
   <si>
@@ -397,9 +385,6 @@
     <t>«Mostrar regras» + medir no F12</t>
   </si>
   <si>
-    <t>N.º de níveis, de 4 (título &gt; promessa &gt; corpo &gt; rodapé), cada um ≥ 1,2× o seguinte</t>
-  </si>
-  <si>
     <t>Ler os tamanhos no F12 (Computed)</t>
   </si>
   <si>
@@ -421,27 +406,6 @@
     <t>Procurar #A8600F no CSS e na página</t>
   </si>
   <si>
-    <t>Desvio da proporção imagem:texto em relação a 2:1 (8:4 colunas)</t>
-  </si>
-  <si>
-    <t>&gt; 30 %</t>
-  </si>
-  <si>
-    <t>21–30 %</t>
-  </si>
-  <si>
-    <t>11–20 %</t>
-  </si>
-  <si>
-    <t>6–10 %</t>
-  </si>
-  <si>
-    <t>≤ 5 %</t>
-  </si>
-  <si>
-    <t>Medir as larguras no F12</t>
-  </si>
-  <si>
     <t>Menor espaço entre secções (px)</t>
   </si>
   <si>
@@ -625,27 +589,18 @@
     <t>1. Cada critério tem uma medida numérica (px, s, %, contagem, pontuação). Mede-se com o instrumento da coluna «Como testar».</t>
   </si>
   <si>
-    <t>2. Escolhe-se o nível (0/25/50/75/100) onde cai o valor medido e escreve-se na coluna azul da folha QEF.</t>
-  </si>
-  <si>
     <t>3. O q (%) calcula-se sozinho. Medições a 1280 px de largura, salvo indicação.</t>
   </si>
   <si>
     <t>4. Quem avalia não é quem fez a regra (revisão cruzada).</t>
   </si>
   <si>
-    <t>Teste com utilizadores (UF1–UF3 e FC4)</t>
-  </si>
-  <si>
     <t>3–5 pessoas que não fizeram a página, sem ajuda, com cronómetro.</t>
   </si>
   <si>
     <t>Tarefa 1: encontrar as lições do curso. Tarefa 2: mostrar as regras e dizer onde está aplicada a regra n.º 3. Tarefa 3: voltar a esconder as regras.</t>
   </si>
   <si>
-    <t>Depois: 2 min com «Mostrar regras» ligado; cada pessoa diz que regra ilustra cada marcador (FC4). No fim, questionário SUS (10 perguntas, escala 1–5).</t>
-  </si>
-  <si>
     <t>FI4 - As setas passam de regra em regra</t>
   </si>
   <si>
@@ -683,6 +638,42 @@
   </si>
   <si>
     <t>5. E03 e UA4: o Lighthouse só analisa páginas http/https, não o ficheiro aberto com duplo clique. Na pasta Files/Teoricas, correr npx http-server e abrir http://localhost:8080/ComposicaoVisual_Pagina_Estatica_Grupo1.html. O E01 continua a medir-se com duplo clique.</t>
+  </si>
+  <si>
+    <t>2. Escolhe-se o nível (0/25/50/75/100) onde cai o valor medido e escreve-se na coluna amarela (J) da folha QEF.</t>
+  </si>
+  <si>
+    <t>Teste com utilizadores (UF1–UF3, FC4 e EC5)</t>
+  </si>
+  <si>
+    <t>Depois: com as regras escondidas, pergunta-se «A abertura pende para algum lado?» (EC5). A seguir, 2 min com «Mostrar regras» ligado; cada pessoa diz que regra ilustra cada marcador (FC4). No fim, questionário SUS (10 perguntas, escala 1–5).</t>
+  </si>
+  <si>
+    <t>N.º de pares seguidos, de 3 (título/promessa, promessa/corpo, corpo/rodapé), em que o maior é ≥ 1,2× o menor</t>
+  </si>
+  <si>
+    <t>N.º de condições, de 3: proporção foto:texto a ≤ 10 % de 2:1 (8:4 colunas) · ≥ 1/3 da altura da abertura vazia do lado do texto · ≥ 80 % das pessoas do teste dizem que a abertura não pende para nenhum lado</t>
+  </si>
+  <si>
+    <t>Medir larguras e alturas no F12; pergunta no teste com utilizadores (ver Notas)</t>
+  </si>
+  <si>
+    <t>&gt; 6 s e ≤ 10 s</t>
+  </si>
+  <si>
+    <t>&gt; 3 s e ≤ 6 s</t>
+  </si>
+  <si>
+    <t>&lt; 4</t>
+  </si>
+  <si>
+    <t>≥ 4 e &lt; 6</t>
+  </si>
+  <si>
+    <t>≥ 6 e &lt; 8</t>
+  </si>
+  <si>
+    <t>≥ 8 e &lt; 10</t>
   </si>
 </sst>
 </file>
@@ -858,10 +849,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -870,10 +858,13 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1260,29 +1251,29 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="22">
+      <c r="A2" s="26">
         <f>(1-B2/SQRT(4))*100</f>
         <v>0</v>
       </c>
-      <c r="B2" s="24">
+      <c r="B2" s="23">
         <f>SQRT((1-C2/100)^2+(1-C10/100)^2+(1-C14/100)^2+(1-C25/100)^2)</f>
         <v>2</v>
       </c>
-      <c r="C2" s="24">
+      <c r="C2" s="23">
         <f>SUMPRODUCT(E2:E9,F2:F9)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="24">
+      <c r="E2" s="23">
         <f>(1/SUM(H2:H5))*SUMPRODUCT(H2:H5,J2:J5)</f>
         <v>0</v>
       </c>
-      <c r="F2" s="26">
+      <c r="F2" s="22">
         <v>0.4</v>
       </c>
-      <c r="G2" s="26" t="s">
+      <c r="G2" s="22" t="s">
         <v>16</v>
       </c>
       <c r="H2" s="3">
@@ -1299,13 +1290,13 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="22"/>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
+      <c r="A3" s="26"/>
+      <c r="B3" s="23"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
       <c r="H3" s="3">
         <v>8</v>
       </c>
@@ -1320,13 +1311,13 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="27"/>
+      <c r="A4" s="27"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
       <c r="H4" s="15">
         <v>6</v>
       </c>
@@ -1341,18 +1332,18 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="22"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
+      <c r="A5" s="26"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
       <c r="H5" s="3">
         <v>6</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="J5" s="4">
         <v>0</v>
@@ -1362,18 +1353,18 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="22"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="26"/>
-      <c r="E6" s="24">
+      <c r="A6" s="26"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23">
         <f>(1/SUM(H6:H9))*SUMPRODUCT(H6:H9,J6:J9)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="22">
         <v>0.6</v>
       </c>
-      <c r="G6" s="26" t="s">
+      <c r="G6" s="22" t="s">
         <v>21</v>
       </c>
       <c r="H6" s="3">
@@ -1390,13 +1381,13 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="22"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="23"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
       <c r="H7" s="3">
         <v>8</v>
       </c>
@@ -1411,13 +1402,13 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="22"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
+      <c r="A8" s="26"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
       <c r="H8" s="3">
         <v>6</v>
       </c>
@@ -1432,13 +1423,13 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="22"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="26"/>
-      <c r="G9" s="26"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
       <c r="H9" s="3">
         <v>8</v>
       </c>
@@ -1453,23 +1444,23 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="22"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24">
+      <c r="A10" s="26"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23">
         <f>SUMPRODUCT(E10:E13,F10:F13)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="23">
         <f>(1/SUM(H10:H13))*SUMPRODUCT(H10:H13,J10:J13)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="22">
         <v>1</v>
       </c>
-      <c r="G10" s="26" t="s">
+      <c r="G10" s="22" t="s">
         <v>27</v>
       </c>
       <c r="H10" s="3">
@@ -1486,13 +1477,13 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="22"/>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="26"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="26"/>
-      <c r="G11" s="26"/>
+      <c r="A11" s="26"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
       <c r="H11" s="3">
         <v>8</v>
       </c>
@@ -1507,13 +1498,13 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="22"/>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
+      <c r="A12" s="26"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
       <c r="H12" s="3">
         <v>8</v>
       </c>
@@ -1528,13 +1519,13 @@
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="22"/>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="26"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="26"/>
-      <c r="G13" s="26"/>
+      <c r="A13" s="26"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
       <c r="H13" s="3">
         <v>6</v>
       </c>
@@ -1549,23 +1540,23 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="22"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24">
+      <c r="A14" s="26"/>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23">
         <f>SUMPRODUCT(E14:E24,F14:F24)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="24">
+      <c r="E14" s="23">
         <f>(1/SUM(H14:H21))*SUMPRODUCT(H14:H21,J14:J21)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="22">
         <v>0.6</v>
       </c>
-      <c r="G14" s="26" t="s">
+      <c r="G14" s="22" t="s">
         <v>36</v>
       </c>
       <c r="H14" s="3">
@@ -1582,13 +1573,13 @@
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="22"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
+      <c r="A15" s="26"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
       <c r="H15" s="3">
         <v>8</v>
       </c>
@@ -1603,13 +1594,13 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="22"/>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
       <c r="H16" s="3">
         <v>8</v>
       </c>
@@ -1624,13 +1615,13 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="22"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="26"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
+      <c r="A17" s="26"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
       <c r="H17" s="3">
         <v>8</v>
       </c>
@@ -1645,13 +1636,13 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="22"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
+      <c r="A18" s="26"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
       <c r="H18" s="3">
         <v>6</v>
       </c>
@@ -1666,13 +1657,13 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="22"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
+      <c r="A19" s="26"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
       <c r="H19" s="3">
         <v>6</v>
       </c>
@@ -1687,13 +1678,13 @@
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="22"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
+      <c r="A20" s="26"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
       <c r="H20" s="3">
         <v>6</v>
       </c>
@@ -1708,13 +1699,13 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="22"/>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="26"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
+      <c r="A21" s="26"/>
+      <c r="B21" s="23"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
       <c r="H21" s="3">
         <v>6</v>
       </c>
@@ -1729,18 +1720,18 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="22"/>
-      <c r="B22" s="24"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="24">
+      <c r="A22" s="26"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="23">
         <f>(1/SUM(H22:H24))*SUMPRODUCT(H22:H24,J22:J24)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="26">
+      <c r="F22" s="22">
         <v>0.4</v>
       </c>
-      <c r="G22" s="26" t="s">
+      <c r="G22" s="22" t="s">
         <v>40</v>
       </c>
       <c r="H22" s="3">
@@ -1757,13 +1748,13 @@
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="22"/>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="26"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="26"/>
+      <c r="A23" s="26"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="22"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
       <c r="H23" s="3">
         <v>10</v>
       </c>
@@ -1778,13 +1769,13 @@
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="22"/>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="26"/>
-      <c r="G24" s="26"/>
+      <c r="A24" s="26"/>
+      <c r="B24" s="23"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
       <c r="H24" s="3">
         <v>8</v>
       </c>
@@ -1799,23 +1790,23 @@
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="22"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="24">
+      <c r="A25" s="26"/>
+      <c r="B25" s="23"/>
+      <c r="C25" s="23">
         <f>SUMPRODUCT(E25:E32,F25:F32)</f>
         <v>0</v>
       </c>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="E25" s="24">
+      <c r="E25" s="23">
         <f>(1/SUM(H25:H27))*SUMPRODUCT(H25:H27,J25:J27)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="22">
         <v>0.4</v>
       </c>
-      <c r="G25" s="26" t="s">
+      <c r="G25" s="22" t="s">
         <v>45</v>
       </c>
       <c r="H25" s="3">
@@ -1832,13 +1823,13 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="22"/>
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="26"/>
+      <c r="A26" s="26"/>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
       <c r="H26" s="3">
         <v>8</v>
       </c>
@@ -1853,13 +1844,13 @@
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="22"/>
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="26"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
+      <c r="A27" s="26"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
       <c r="H27" s="3">
         <v>8</v>
       </c>
@@ -1874,18 +1865,18 @@
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="22"/>
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="24">
+      <c r="A28" s="26"/>
+      <c r="B28" s="23"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="23">
         <f>(1/SUM(H28:H31))*SUMPRODUCT(H28:H31,J28:J31)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="26">
+      <c r="F28" s="22">
         <v>0.4</v>
       </c>
-      <c r="G28" s="26" t="s">
+      <c r="G28" s="22" t="s">
         <v>50</v>
       </c>
       <c r="H28" s="3">
@@ -1902,13 +1893,13 @@
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="22"/>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="26"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="26"/>
-      <c r="G29" s="26"/>
+      <c r="A29" s="26"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="22"/>
       <c r="H29" s="3">
         <v>8</v>
       </c>
@@ -1923,13 +1914,13 @@
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="22"/>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="26"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
+      <c r="A30" s="26"/>
+      <c r="B30" s="23"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="22"/>
       <c r="H30" s="3">
         <v>6</v>
       </c>
@@ -1944,13 +1935,13 @@
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="22"/>
-      <c r="B31" s="24"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="26"/>
-      <c r="G31" s="26"/>
+      <c r="A31" s="26"/>
+      <c r="B31" s="23"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="22"/>
       <c r="H31" s="3">
         <v>6</v>
       </c>
@@ -1965,10 +1956,10 @@
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="22"/>
-      <c r="B32" s="24"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="26"/>
+      <c r="A32" s="26"/>
+      <c r="B32" s="23"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="22"/>
       <c r="E32" s="5">
         <f>(1/SUM(H32:H32))*SUMPRODUCT(H32:H32,J32:J32)</f>
         <v>0</v>
@@ -1994,26 +1985,6 @@
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="G10:G13"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="G2:G5"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="G6:G9"/>
-    <mergeCell ref="F14:F21"/>
-    <mergeCell ref="G14:G21"/>
-    <mergeCell ref="E22:E24"/>
-    <mergeCell ref="F22:F24"/>
-    <mergeCell ref="G22:G24"/>
-    <mergeCell ref="F25:F27"/>
-    <mergeCell ref="G25:G27"/>
-    <mergeCell ref="E28:E31"/>
-    <mergeCell ref="F28:F31"/>
-    <mergeCell ref="G28:G31"/>
     <mergeCell ref="A2:A32"/>
     <mergeCell ref="B2:B32"/>
     <mergeCell ref="C14:C24"/>
@@ -2025,6 +1996,26 @@
     <mergeCell ref="C2:C9"/>
     <mergeCell ref="D2:D9"/>
     <mergeCell ref="E10:E13"/>
+    <mergeCell ref="F25:F27"/>
+    <mergeCell ref="G25:G27"/>
+    <mergeCell ref="E28:E31"/>
+    <mergeCell ref="F28:F31"/>
+    <mergeCell ref="G28:G31"/>
+    <mergeCell ref="F14:F21"/>
+    <mergeCell ref="G14:G21"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="F22:F24"/>
+    <mergeCell ref="G22:G24"/>
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="G10:G13"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="G2:G5"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="G6:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2095,25 +2086,25 @@
         <v>12</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="D5" s="18" t="s">
         <v>89</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="G5" s="18" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -2176,13 +2167,13 @@
     </row>
     <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="B8" s="20" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="D8" s="21">
         <v>0</v>
@@ -2200,7 +2191,7 @@
         <v>4</v>
       </c>
       <c r="I8" s="19" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -2338,22 +2329,22 @@
         <v>88</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>89</v>
+        <v>206</v>
       </c>
       <c r="E16" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="H16" s="11">
+        <v>10</v>
+      </c>
+      <c r="I16" s="8" t="s">
         <v>90</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>91</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -2426,25 +2417,25 @@
         <v>14</v>
       </c>
       <c r="C5" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="E5" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="F5" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="G5" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="H5" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="I5" s="8" t="s">
         <v>97</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -2455,7 +2446,7 @@
         <v>14</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>69</v>
@@ -2473,7 +2464,7 @@
         <v>60</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -2484,25 +2475,25 @@
         <v>14</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="G7" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="H7" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="E7" s="11" t="s">
-        <v>104</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>105</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>107</v>
-      </c>
       <c r="I7" s="8" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -2513,7 +2504,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>69</v>
@@ -2531,7 +2522,7 @@
         <v>58</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -2604,28 +2595,28 @@
         <v>12</v>
       </c>
       <c r="C5" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="H5" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="I5" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="F5" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>29</v>
       </c>
@@ -2633,25 +2624,23 @@
         <v>12</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>117</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>59</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="H6" s="11" t="s">
-        <v>60</v>
+        <v>201</v>
+      </c>
+      <c r="D6" s="11">
+        <v>0</v>
+      </c>
+      <c r="E6" s="11">
+        <v>1</v>
+      </c>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11">
+        <v>2</v>
+      </c>
+      <c r="H6" s="11">
+        <v>3</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -2662,10 +2651,10 @@
         <v>12</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>75</v>
@@ -2680,7 +2669,7 @@
         <v>69</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -2691,10 +2680,10 @@
         <v>12</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>59</v>
@@ -2709,10 +2698,10 @@
         <v>69</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>32</v>
       </c>
@@ -2720,25 +2709,23 @@
         <v>12</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="H9" s="11" t="s">
-        <v>130</v>
+        <v>202</v>
+      </c>
+      <c r="D9" s="11">
+        <v>0</v>
+      </c>
+      <c r="E9" s="11">
+        <v>1</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11">
+        <v>2</v>
+      </c>
+      <c r="H9" s="11">
+        <v>3</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>131</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -2749,25 +2736,25 @@
         <v>12</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>134</v>
+        <v>122</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>135</v>
+        <v>123</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="H10" s="11" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -2778,10 +2765,10 @@
         <v>12</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>139</v>
+        <v>127</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>59</v>
@@ -2796,7 +2783,7 @@
         <v>69</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>140</v>
+        <v>128</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -2807,7 +2794,7 @@
         <v>12</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>69</v>
@@ -2825,7 +2812,7 @@
         <v>60</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
@@ -2873,10 +2860,10 @@
         <v>14</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="D17" s="11" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>59</v>
@@ -2891,7 +2878,7 @@
         <v>69</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -2902,7 +2889,7 @@
         <v>14</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>69</v>
@@ -2920,7 +2907,7 @@
         <v>60</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -2931,7 +2918,7 @@
         <v>14</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>62</v>
@@ -2949,7 +2936,7 @@
         <v>66</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>148</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -3022,25 +3009,25 @@
         <v>14</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>149</v>
+        <v>137</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>151</v>
+        <v>139</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>66</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -3051,25 +3038,25 @@
         <v>14</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -3080,25 +3067,25 @@
         <v>14</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3146,7 +3133,7 @@
         <v>14</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>62</v>
@@ -3164,7 +3151,7 @@
         <v>66</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -3175,25 +3162,25 @@
         <v>14</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>66</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -3204,10 +3191,10 @@
         <v>14</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>59</v>
@@ -3222,7 +3209,7 @@
         <v>69</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -3233,25 +3220,25 @@
         <v>14</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -3299,7 +3286,7 @@
         <v>14</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>69</v>
@@ -3317,7 +3304,7 @@
         <v>60</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -3335,7 +3322,7 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -3343,17 +3330,17 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
@@ -3361,17 +3348,17 @@
     </row>
     <row r="7" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -3379,32 +3366,32 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>194</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>195</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:1" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -3412,22 +3399,22 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>197</v>
+        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Recursos para a liçao 4 e atualizacao da composicao visual da plataforma html
</commit_message>
<xml_diff>
--- a/Files/Teoricas/ComposicaoVisual_QEF_Grupo1.xlsx
+++ b/Files/Teoricas/ComposicaoVisual_QEF_Grupo1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tiago\AppData\Local\Temp\claude\C--Users-tiago-Desktop-Mestrado-2Ano-CAMUL-RepoCamul-CAMUL-2026\67b76cae-61ff-4d41-a191-a6d9f77c0f89\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Mestrado-Jogos\CAMUL\CAMUL-2026\Files\Teoricas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E86D98A-5DCE-4E56-8EF4-37B2C1776948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B0821B-5117-4118-9117-D0DFCF039B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2BE1A5F0-6062-45CC-8E94-69B694959B5C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{2BE1A5F0-6062-45CC-8E94-69B694959B5C}"/>
   </bookViews>
   <sheets>
     <sheet name="QEF" sheetId="1" r:id="rId1"/>
@@ -786,7 +786,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -840,16 +840,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -858,13 +852,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1251,29 +1242,29 @@
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="26">
+      <c r="A2" s="19">
         <f>(1-B2/SQRT(4))*100</f>
         <v>0</v>
       </c>
-      <c r="B2" s="23">
+      <c r="B2" s="21">
         <f>SQRT((1-C2/100)^2+(1-C10/100)^2+(1-C14/100)^2+(1-C25/100)^2)</f>
         <v>2</v>
       </c>
-      <c r="C2" s="23">
+      <c r="C2" s="21">
         <f>SUMPRODUCT(E2:E9,F2:F9)</f>
         <v>0</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="23">
+      <c r="E2" s="21">
         <f>(1/SUM(H2:H5))*SUMPRODUCT(H2:H5,J2:J5)</f>
         <v>0</v>
       </c>
-      <c r="F2" s="22">
+      <c r="F2" s="23">
         <v>0.4</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="23" t="s">
         <v>16</v>
       </c>
       <c r="H2" s="3">
@@ -1290,13 +1281,13 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="26"/>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="23"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
+      <c r="A3" s="19"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
       <c r="H3" s="3">
         <v>8</v>
       </c>
@@ -1311,13 +1302,13 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="27"/>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
       <c r="H4" s="15">
         <v>6</v>
       </c>
@@ -1332,13 +1323,13 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="23"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
+      <c r="A5" s="19"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="23"/>
+      <c r="G5" s="23"/>
       <c r="H5" s="3">
         <v>6</v>
       </c>
@@ -1353,18 +1344,18 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="26"/>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="23">
+      <c r="A6" s="19"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="23"/>
+      <c r="E6" s="21">
         <f>(1/SUM(H6:H9))*SUMPRODUCT(H6:H9,J6:J9)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="23">
         <v>0.6</v>
       </c>
-      <c r="G6" s="22" t="s">
+      <c r="G6" s="23" t="s">
         <v>21</v>
       </c>
       <c r="H6" s="3">
@@ -1381,13 +1372,13 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="26"/>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="22"/>
-      <c r="E7" s="23"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
+      <c r="A7" s="19"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="23"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="23"/>
       <c r="H7" s="3">
         <v>8</v>
       </c>
@@ -1402,13 +1393,13 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="26"/>
-      <c r="B8" s="23"/>
-      <c r="C8" s="23"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
+      <c r="A8" s="19"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="23"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="23"/>
+      <c r="G8" s="23"/>
       <c r="H8" s="3">
         <v>6</v>
       </c>
@@ -1423,13 +1414,13 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="26"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
+      <c r="A9" s="19"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="23"/>
+      <c r="G9" s="23"/>
       <c r="H9" s="3">
         <v>8</v>
       </c>
@@ -1444,23 +1435,23 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="26"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23">
+      <c r="A10" s="19"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21">
         <f>SUMPRODUCT(E10:E13,F10:F13)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="21">
         <f>(1/SUM(H10:H13))*SUMPRODUCT(H10:H13,J10:J13)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="23">
         <v>1</v>
       </c>
-      <c r="G10" s="22" t="s">
+      <c r="G10" s="23" t="s">
         <v>27</v>
       </c>
       <c r="H10" s="3">
@@ -1477,13 +1468,13 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="26"/>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
+      <c r="A11" s="19"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
       <c r="H11" s="3">
         <v>8</v>
       </c>
@@ -1498,13 +1489,13 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="26"/>
-      <c r="B12" s="23"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="23"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
+      <c r="A12" s="19"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="23"/>
       <c r="H12" s="3">
         <v>8</v>
       </c>
@@ -1519,13 +1510,13 @@
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="26"/>
-      <c r="B13" s="23"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
+      <c r="A13" s="19"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="23"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
       <c r="H13" s="3">
         <v>6</v>
       </c>
@@ -1540,23 +1531,23 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="26"/>
-      <c r="B14" s="23"/>
-      <c r="C14" s="23">
+      <c r="A14" s="19"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21">
         <f>SUMPRODUCT(E14:E24,F14:F24)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E14" s="21">
         <f>(1/SUM(H14:H21))*SUMPRODUCT(H14:H21,J14:J21)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="23">
         <v>0.6</v>
       </c>
-      <c r="G14" s="22" t="s">
+      <c r="G14" s="23" t="s">
         <v>36</v>
       </c>
       <c r="H14" s="3">
@@ -1573,13 +1564,13 @@
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="26"/>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
+      <c r="A15" s="19"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="23"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="23"/>
       <c r="H15" s="3">
         <v>8</v>
       </c>
@@ -1594,13 +1585,13 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="26"/>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
+      <c r="A16" s="19"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
       <c r="H16" s="3">
         <v>8</v>
       </c>
@@ -1615,13 +1606,13 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="26"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
+      <c r="A17" s="19"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
       <c r="H17" s="3">
         <v>8</v>
       </c>
@@ -1636,13 +1627,13 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="26"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
+      <c r="A18" s="19"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="23"/>
       <c r="H18" s="3">
         <v>6</v>
       </c>
@@ -1657,13 +1648,13 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="26"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
+      <c r="A19" s="19"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="23"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
       <c r="H19" s="3">
         <v>6</v>
       </c>
@@ -1678,13 +1669,13 @@
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="26"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
+      <c r="A20" s="19"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
       <c r="H20" s="3">
         <v>6</v>
       </c>
@@ -1699,13 +1690,13 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="26"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
+      <c r="A21" s="19"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
       <c r="H21" s="3">
         <v>6</v>
       </c>
@@ -1720,18 +1711,18 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="26"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="23">
+      <c r="A22" s="19"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="21">
         <f>(1/SUM(H22:H24))*SUMPRODUCT(H22:H24,J22:J24)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="22">
+      <c r="F22" s="23">
         <v>0.4</v>
       </c>
-      <c r="G22" s="22" t="s">
+      <c r="G22" s="23" t="s">
         <v>40</v>
       </c>
       <c r="H22" s="3">
@@ -1748,13 +1739,13 @@
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="26"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="23"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
+      <c r="A23" s="19"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="23"/>
+      <c r="G23" s="23"/>
       <c r="H23" s="3">
         <v>10</v>
       </c>
@@ -1769,13 +1760,13 @@
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="26"/>
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
+      <c r="A24" s="19"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="23"/>
+      <c r="G24" s="23"/>
       <c r="H24" s="3">
         <v>8</v>
       </c>
@@ -1790,23 +1781,23 @@
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="26"/>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23">
+      <c r="A25" s="19"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21">
         <f>SUMPRODUCT(E25:E32,F25:F32)</f>
         <v>0</v>
       </c>
-      <c r="D25" s="22" t="s">
+      <c r="D25" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="E25" s="23">
+      <c r="E25" s="21">
         <f>(1/SUM(H25:H27))*SUMPRODUCT(H25:H27,J25:J27)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="22">
+      <c r="F25" s="23">
         <v>0.4</v>
       </c>
-      <c r="G25" s="22" t="s">
+      <c r="G25" s="23" t="s">
         <v>45</v>
       </c>
       <c r="H25" s="3">
@@ -1823,13 +1814,13 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="26"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
+      <c r="A26" s="19"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="23"/>
       <c r="H26" s="3">
         <v>8</v>
       </c>
@@ -1844,13 +1835,13 @@
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="26"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
+      <c r="A27" s="19"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="23"/>
       <c r="H27" s="3">
         <v>8</v>
       </c>
@@ -1865,18 +1856,18 @@
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="26"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="23">
+      <c r="A28" s="19"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="21">
         <f>(1/SUM(H28:H31))*SUMPRODUCT(H28:H31,J28:J31)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="22">
+      <c r="F28" s="23">
         <v>0.4</v>
       </c>
-      <c r="G28" s="22" t="s">
+      <c r="G28" s="23" t="s">
         <v>50</v>
       </c>
       <c r="H28" s="3">
@@ -1893,13 +1884,13 @@
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="26"/>
-      <c r="B29" s="23"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="22"/>
+      <c r="A29" s="19"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="23"/>
       <c r="H29" s="3">
         <v>8</v>
       </c>
@@ -1914,13 +1905,13 @@
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="26"/>
-      <c r="B30" s="23"/>
-      <c r="C30" s="23"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
+      <c r="A30" s="19"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="23"/>
       <c r="H30" s="3">
         <v>6</v>
       </c>
@@ -1935,13 +1926,13 @@
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="26"/>
-      <c r="B31" s="23"/>
-      <c r="C31" s="23"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="22"/>
-      <c r="G31" s="22"/>
+      <c r="A31" s="19"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="23"/>
       <c r="H31" s="3">
         <v>6</v>
       </c>
@@ -1956,10 +1947,10 @@
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="26"/>
-      <c r="B32" s="23"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="22"/>
+      <c r="A32" s="19"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="23"/>
       <c r="E32" s="5">
         <f>(1/SUM(H32:H32))*SUMPRODUCT(H32:H32,J32:J32)</f>
         <v>0</v>
@@ -1985,6 +1976,26 @@
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="F10:F13"/>
+    <mergeCell ref="G10:G13"/>
+    <mergeCell ref="C10:C13"/>
+    <mergeCell ref="D10:D13"/>
+    <mergeCell ref="E2:E5"/>
+    <mergeCell ref="F2:F5"/>
+    <mergeCell ref="G2:G5"/>
+    <mergeCell ref="E6:E9"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="G6:G9"/>
+    <mergeCell ref="F14:F21"/>
+    <mergeCell ref="G14:G21"/>
+    <mergeCell ref="E22:E24"/>
+    <mergeCell ref="F22:F24"/>
+    <mergeCell ref="G22:G24"/>
+    <mergeCell ref="F25:F27"/>
+    <mergeCell ref="G25:G27"/>
+    <mergeCell ref="E28:E31"/>
+    <mergeCell ref="F28:F31"/>
+    <mergeCell ref="G28:G31"/>
     <mergeCell ref="A2:A32"/>
     <mergeCell ref="B2:B32"/>
     <mergeCell ref="C14:C24"/>
@@ -1996,26 +2007,6 @@
     <mergeCell ref="C2:C9"/>
     <mergeCell ref="D2:D9"/>
     <mergeCell ref="E10:E13"/>
-    <mergeCell ref="F25:F27"/>
-    <mergeCell ref="G25:G27"/>
-    <mergeCell ref="E28:E31"/>
-    <mergeCell ref="F28:F31"/>
-    <mergeCell ref="G28:G31"/>
-    <mergeCell ref="F14:F21"/>
-    <mergeCell ref="G14:G21"/>
-    <mergeCell ref="E22:E24"/>
-    <mergeCell ref="F22:F24"/>
-    <mergeCell ref="G22:G24"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="G10:G13"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="G2:G5"/>
-    <mergeCell ref="E6:E9"/>
-    <mergeCell ref="F6:F9"/>
-    <mergeCell ref="G6:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2166,31 +2157,31 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="75" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="D8" s="21">
-        <v>0</v>
-      </c>
-      <c r="E8" s="21">
+      <c r="D8" s="11">
+        <v>0</v>
+      </c>
+      <c r="E8" s="11">
         <v>1</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="11">
         <v>2</v>
       </c>
-      <c r="G8" s="21">
+      <c r="G8" s="11">
         <v>3</v>
       </c>
-      <c r="H8" s="21">
+      <c r="H8" s="11">
         <v>4</v>
       </c>
-      <c r="I8" s="19" t="s">
+      <c r="I8" s="8" t="s">
         <v>193</v>
       </c>
     </row>

</xml_diff>